<commit_message>
This preprocessing stuff is hard
That is why we're here: to learn.
</commit_message>
<xml_diff>
--- a/Documentation/Compiler Directives.xlsx
+++ b/Documentation/Compiler Directives.xlsx
@@ -716,7 +716,7 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:E77" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="A1:E77"/>
-  <sortState ref="A2:E77">
+  <sortState ref="A13:E32">
     <sortCondition ref="C1:C77"/>
   </sortState>
   <tableColumns count="5">
@@ -1259,7 +1259,7 @@
       <c r="D14" s="8" t="e">
         <v>#N/A</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="1" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1333,27 +1333,27 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B19" t="s">
-        <v>109</v>
+        <v>129</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D19" s="8" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E19" s="2" t="e">
-        <v>#N/A</v>
+      <c r="D19" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>137</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>97</v>
@@ -1361,16 +1361,16 @@
       <c r="D20" s="8" t="e">
         <v>#N/A</v>
       </c>
-      <c r="E20" s="2" t="e">
-        <v>#N/A</v>
+      <c r="E20" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>58</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>97</v>
@@ -1378,22 +1378,22 @@
       <c r="D21" s="8" t="e">
         <v>#N/A</v>
       </c>
-      <c r="E21" s="8" t="e">
-        <v>#N/A</v>
+      <c r="E21" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>76</v>
       </c>
       <c r="B22" t="s">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D22" s="12" t="s">
-        <v>127</v>
+      <c r="D22" s="6">
+        <v>1048576</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>3</v>
@@ -1435,33 +1435,33 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>137</v>
+        <v>52</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D25" s="8" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>3</v>
+      <c r="D25" s="6">
+        <v>1</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>151</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D26" s="6">
-        <v>1</v>
+      <c r="D26" s="8" t="e">
+        <v>#N/A</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>95</v>
@@ -1469,10 +1469,10 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>109</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>97</v>
@@ -1480,16 +1480,16 @@
       <c r="D27" s="8" t="e">
         <v>#N/A</v>
       </c>
-      <c r="E27" s="8" t="e">
+      <c r="E27" s="2" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>97</v>
@@ -1497,16 +1497,16 @@
       <c r="D28" s="8" t="e">
         <v>#N/A</v>
       </c>
-      <c r="E28" s="8" t="e">
+      <c r="E28" s="2" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>58</v>
+        <v>117</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>97</v>
@@ -1514,16 +1514,16 @@
       <c r="D29" s="8" t="e">
         <v>#N/A</v>
       </c>
-      <c r="E29" s="4" t="s">
-        <v>3</v>
+      <c r="E29" s="8" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="B30" t="s">
-        <v>148</v>
+        <v>54</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>97</v>
@@ -1537,27 +1537,27 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="B31" t="s">
-        <v>149</v>
+        <v>56</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="D31" s="6">
-        <v>1048576</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>3</v>
+      <c r="D31" s="8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E31" s="8" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>97</v>
@@ -1565,84 +1565,84 @@
       <c r="D32" s="8" t="e">
         <v>#N/A</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>95</v>
+      <c r="E32" s="8" t="e">
+        <v>#N/A</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>104</v>
+        <v>167</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D33" s="6">
-        <v>8</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>95</v>
+      <c r="D33" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="B34" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>95</v>
+      <c r="D34" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="B35" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>95</v>
+      <c r="D35" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>99</v>
+        <v>128</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D36" s="5">
-        <v>0</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>95</v>
+      <c r="D36" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="B37" t="s">
-        <v>167</v>
+        <v>43</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>2</v>
@@ -1656,50 +1656,50 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="B38" t="s">
-        <v>101</v>
+        <v>135</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D38" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>95</v>
+      <c r="D38" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="B39" t="s">
-        <v>103</v>
+        <v>67</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D39" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>95</v>
+      <c r="D39" s="8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>22</v>
+        <v>83</v>
       </c>
       <c r="B40" t="s">
-        <v>111</v>
+        <v>157</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>3</v>
@@ -1707,10 +1707,10 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="B41" t="s">
-        <v>112</v>
+        <v>158</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>2</v>
@@ -1724,10 +1724,10 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="B42" t="s">
-        <v>113</v>
+        <v>159</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>2</v>
@@ -1735,22 +1735,22 @@
       <c r="D42" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="E42" s="1" t="s">
-        <v>95</v>
+      <c r="E42" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="B43" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D43" s="9" t="s">
-        <v>1</v>
+      <c r="D43" s="6">
+        <v>8</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>95</v>
@@ -1758,16 +1758,16 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="B44" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D44" s="7" t="s">
-        <v>98</v>
+      <c r="D44" s="5" t="s">
+        <v>1</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>95</v>
@@ -1775,16 +1775,16 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B45" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D45" s="9" t="s">
-        <v>1</v>
+      <c r="D45" s="7" t="s">
+        <v>98</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>95</v>
@@ -1792,33 +1792,33 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="B46" t="s">
-        <v>128</v>
+        <v>99</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D46" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>3</v>
+      <c r="D46" s="5">
+        <v>0</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="B47" t="s">
-        <v>130</v>
+        <v>101</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D47" s="9" t="s">
-        <v>1</v>
+      <c r="D47" s="7" t="s">
+        <v>98</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>95</v>
@@ -1826,16 +1826,16 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="B48" t="s">
-        <v>132</v>
+        <v>103</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D48" s="9" t="s">
-        <v>1</v>
+      <c r="D48" s="7" t="s">
+        <v>98</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>95</v>
@@ -1843,27 +1843,27 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="B49" t="s">
-        <v>43</v>
+        <v>113</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>3</v>
+      <c r="D49" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="B50" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>2</v>
@@ -1871,22 +1871,22 @@
       <c r="D50" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E50" s="4" t="s">
-        <v>3</v>
+      <c r="E50" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="B51" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D51" s="9" t="s">
-        <v>1</v>
+      <c r="D51" s="7" t="s">
+        <v>98</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>95</v>
@@ -1894,16 +1894,16 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="B52" t="s">
-        <v>168</v>
+        <v>116</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D52" s="7" t="s">
-        <v>98</v>
+      <c r="D52" s="9" t="s">
+        <v>1</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>95</v>
@@ -1911,10 +1911,10 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="B53" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>2</v>
@@ -1928,10 +1928,10 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="B54" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>2</v>
@@ -1945,16 +1945,16 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="B55" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D55" s="7" t="s">
-        <v>98</v>
+      <c r="D55" s="9" t="s">
+        <v>1</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>95</v>
@@ -1962,33 +1962,33 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="B56" t="s">
-        <v>67</v>
+        <v>168</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D56" s="8" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E56" s="4" t="s">
-        <v>3</v>
+      <c r="D56" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="B57" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D57" s="7" t="s">
-        <v>98</v>
+      <c r="D57" s="9" t="s">
+        <v>1</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>95</v>
@@ -1996,16 +1996,16 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B58" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D58" s="7" t="s">
-        <v>98</v>
+      <c r="D58" s="9" t="s">
+        <v>1</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>95</v>
@@ -2013,10 +2013,10 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B59" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>2</v>
@@ -2030,10 +2030,10 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B60" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>2</v>
@@ -2047,10 +2047,10 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B61" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>2</v>
@@ -2064,10 +2064,10 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B62" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>2</v>
@@ -2081,10 +2081,10 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B63" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>2</v>
@@ -2098,10 +2098,10 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B64" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>2</v>
@@ -2115,10 +2115,10 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B65" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>2</v>
@@ -2126,33 +2126,33 @@
       <c r="D65" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="E65" s="4" t="s">
-        <v>3</v>
+      <c r="E65" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B66" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D66" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E66" s="4" t="s">
-        <v>3</v>
+      <c r="D66" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B67" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>2</v>
@@ -2160,8 +2160,8 @@
       <c r="D67" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="E67" s="4" t="s">
-        <v>3</v>
+      <c r="E67" s="1" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="68" spans="1:5">

</xml_diff>